<commit_message>
Deeplink suite with login prep, separate verification, and local build/install
</commit_message>
<xml_diff>
--- a/testcases/deeplinks/deeplink_tests.xlsx
+++ b/testcases/deeplinks/deeplink_tests.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marnisaisanjay/Documents/personalprojects/AppPilot/testcases/deeplinks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD93778B-B596-3940-BC60-B81373E8F6B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95D637E8-0406-0140-8BE7-D18AB3CCDD3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{C5943666-9D12-0C47-8784-2B49B0DE6ECC}"/>
   </bookViews>
@@ -39,48 +39,57 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="17">
+  <si>
+    <t>Premium</t>
+  </si>
+  <si>
+    <t>Test Case ID</t>
+  </si>
+  <si>
+    <t>Launch URL</t>
+  </si>
+  <si>
+    <t>License</t>
+  </si>
+  <si>
+    <t>Expected Screen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://m365.cloud.microsoft/chat/entity1-d870f6cd-4aa5-4d42-9626-ab690c041429/eyJpZCI6IlRXbGpjbTl6YjJaMFZqSjhhSFIwY0hNNkx5OXpkV0p6ZEhKaGRHVXViMlptYVdObExtTnZiWHd5T1dNM04yTmtNeTFsWldJekxUUmhOekV0T1dFelppMDNaRGt6WWpRME9EQXhZako4WlRRMU16RXlaamN0Tm1Fd01DMDBPVFl5TFdGaE0yWXRNekUzWldFMU1qWmlORFJpZkdWdUxYVnoiLCJzY2VuYXJpbyI6InNoYXJlTGluayIsImNoYXRUeXBlIjoid2ViIiwicHJvcGVydGllcyI6eyJwcm9tcHRTb3VyY2UiOiJtaWNyb3NvZnQiLCJjbGlja1RpbWVzdGFtcCI6IjIwMjYtMDgtMDhUMjE6MzQ6MTYuODU5WiJ9LCJyZWZlcnJhbCI6eyJjbW1pZCI6ImNtbTEyMjIyMjIyIn0sImNvcnJlbGF0aW9uSWQiOiJjZTc2MmM5Zi04ODM4LTRkMzUtODAxMy0xNDk2OTIzNWEzNGIiLCJ2ZXJzaW9uIjoxLjB9?fromcode=cmm12222222&amp;ct=new&amp;ocid=new&amp;utm_campaign=new&amp;utm_source=new </t>
+  </si>
+  <si>
+    <t>Installed</t>
+  </si>
+  <si>
+    <t>Test Case Reference Details</t>
+  </si>
+  <si>
+    <t>TC003</t>
+  </si>
+  <si>
+    <t>no</t>
+  </si>
+  <si>
+    <t>Chat screen with prompt "Summarize the top three news from today, highlighting the main events and their implications. Include any significant developments or updates"</t>
+  </si>
   <si>
     <t>TC001</t>
   </si>
   <si>
-    <t>Premium</t>
-  </si>
-  <si>
-    <t>Chat screen with prompt</t>
-  </si>
-  <si>
     <t>TC002</t>
   </si>
   <si>
-    <t>https://m365.cloud.microsoft/?openAppStoreOnLoad=true&amp;fromcode=cmm12222222&amp;referrer=utm_source%3Dnew%26utm_campaign%3Dnew&amp;ocid=new&amp;pt=80423&amp;ct=new&amp;qrversion=email&amp;ccac=tofqrcode</t>
-  </si>
-  <si>
-    <t>Chat screen</t>
-  </si>
-  <si>
-    <t>Test Case ID</t>
-  </si>
-  <si>
-    <t>Launch URL</t>
-  </si>
-  <si>
-    <t>License</t>
-  </si>
-  <si>
-    <t>Expected Screen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://m365.cloud.microsoft/chat/entity1-d870f6cd-4aa5-4d42-9626-ab690c041429/eyJpZCI6IlRXbGpjbTl6YjJaMFZqSjhhSFIwY0hNNkx5OXpkV0p6ZEhKaGRHVXViMlptYVdObExtTnZiWHd5T1dNM04yTmtNeTFsWldJekxUUmhOekV0T1dFelppMDNaRGt6WWpRME9EQXhZako4WlRRMU16RXlaamN0Tm1Fd01DMDBPVFl5TFdGaE0yWXRNekUzWldFMU1qWmlORFJpZkdWdUxYVnoiLCJzY2VuYXJpbyI6InNoYXJlTGluayIsImNoYXRUeXBlIjoid2ViIiwicHJvcGVydGllcyI6eyJwcm9tcHRTb3VyY2UiOiJtaWNyb3NvZnQiLCJjbGlja1RpbWVzdGFtcCI6IjIwMjYtMDgtMDhUMjE6MzQ6MTYuODU5WiJ9LCJyZWZlcnJhbCI6eyJjbW1pZCI6ImNtbTEyMjIyMjIyIn0sImNvcnJlbGF0aW9uSWQiOiJjZTc2MmM5Zi04ODM4LTRkMzUtODAxMy0xNDk2OTIzNWEzNGIiLCJ2ZXJzaW9uIjoxLjB9?fromcode=cmm12222222&amp;ct=new&amp;ocid=new&amp;utm_campaign=new&amp;utm_source=new </t>
-  </si>
-  <si>
-    <t>Installed</t>
-  </si>
-  <si>
-    <t>yes</t>
-  </si>
-  <si>
-    <t>Test Case Reference Details</t>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>https://m365.cloud.microsoft/?openAppStoreOnLoad=true&amp;fromcode=cmmtest1222&amp;referrer=utm_source%3Dq%26utm_campaign%3Dq&amp;ocid=q&amp;pt=80423&amp;ct=q&amp;qrversion=email&amp;ccac=tofqrcode</t>
+  </si>
+  <si>
+    <t>TC004</t>
+  </si>
+  <si>
+    <t>Chat screen with no prompt</t>
   </si>
 </sst>
 </file>
@@ -118,7 +127,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -126,11 +135,22 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -138,7 +158,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -180,19 +203,15 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C3E0EAF0-8322-9943-9361-9A2C145B69AC}" name="TestCasesTable" displayName="TestCasesTable" ref="A2:E4" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C3E0EAF0-8322-9943-9361-9A2C145B69AC}" name="TestCasesTable" displayName="TestCasesTable" ref="A2:E4" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
   <autoFilter ref="A2:E4" xr:uid="{C3E0EAF0-8322-9943-9361-9A2C145B69AC}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{E7C93395-3D2D-F24C-B14C-2E0B10E9B5B2}" name="Test Case ID" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{1C1E9B71-D984-1A45-98E8-18E5C9778295}" name="Launch URL" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{6CC5405F-8922-2E4C-B7D1-5D204DC658A0}" name="License" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{F4FB8A81-E7AB-BA43-8829-4FE851CDEED2}" name="Expected Screen" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{0D6DC78D-E6A7-C946-892F-2EF1D0741508}" name="Installed" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{E7C93395-3D2D-F24C-B14C-2E0B10E9B5B2}" name="Test Case ID" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{1C1E9B71-D984-1A45-98E8-18E5C9778295}" name="Launch URL" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{6CC5405F-8922-2E4C-B7D1-5D204DC658A0}" name="License" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{F4FB8A81-E7AB-BA43-8829-4FE851CDEED2}" name="Expected Screen" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{0D6DC78D-E6A7-C946-892F-2EF1D0741508}" name="Installed" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -515,7 +534,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B78DF14-4F71-D549-86BA-243B67A56556}">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="34.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="34.6640625" style="1"/>
@@ -524,63 +543,97 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
+      <c r="A1" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
     </row>
     <row r="2" spans="1:5" s="2" customFormat="1" ht="71" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E2" s="2" t="s">
+    </row>
+    <row r="3" spans="1:5" s="2" customFormat="1" ht="71" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" s="2" customFormat="1" ht="123" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="2" t="s">
+      <c r="B3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>2</v>
-      </c>
       <c r="E3" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="2" customFormat="1" ht="71" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D4" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" s="2" customFormat="1" ht="123" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>12</v>
+      <c r="C5" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" s="2" customFormat="1" ht="71" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -588,11 +641,13 @@
     <mergeCell ref="A1:E1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B3" r:id="rId1" display="https://m365.cloud.microsoft/chat/entity1-d870f6cd-4aa5-4d42-9626-ab690c041429/eyJpZCI6IlRXbGpjbTl6YjJaMFZqSjhhSFIwY0hNNkx5OXpkV0p6ZEhKaGRHVXViMlptYVdObExtTnZiWHd5T1dNM04yTmtNeTFsWldJekxUUmhOekV0T1dFelppMDNaRGt6WWpRME9EQXhZako4WlRRMU16RXlaamN0Tm1Fd01DMDBPVFl5TFdGaE0yWXRNekUzWldFMU1qWmlORFJpZkdWdUxYVnoiLCJzY2VuYXJpbyI6InNoYXJlTGluayIsImNoYXRUeXBlIjoid2ViIiwicHJvcGVydGllcyI6eyJwcm9tcHRTb3VyY2UiOiJtaWNyb3NvZnQiLCJjbGlja1RpbWVzdGFtcCI6IjIwMjYtMDgtMDhUMjE6MzQ6MTYuODU5WiJ9LCJyZWZlcnJhbCI6eyJjbW1pZCI6ImNtbTEyMjIyMjIyIn0sImNvcnJlbGF0aW9uSWQiOiJjZTc2MmM5Zi04ODM4LTRkMzUtODAxMy0xNDk2OTIzNWEzNGIiLCJ2ZXJzaW9uIjoxLjB9?fromcode=cmm12222222&amp;ct=new&amp;ocid=new&amp;utm_campaign=new&amp;utm_source=new " xr:uid="{8166E9EC-2AA3-004D-96F9-8E31355B987F}"/>
+    <hyperlink ref="B5" r:id="rId1" display="https://m365.cloud.microsoft/chat/entity1-d870f6cd-4aa5-4d42-9626-ab690c041429/eyJpZCI6IlRXbGpjbTl6YjJaMFZqSjhhSFIwY0hNNkx5OXpkV0p6ZEhKaGRHVXViMlptYVdObExtTnZiWHd5T1dNM04yTmtNeTFsWldJekxUUmhOekV0T1dFelppMDNaRGt6WWpRME9EQXhZako4WlRRMU16RXlaamN0Tm1Fd01DMDBPVFl5TFdGaE0yWXRNekUzWldFMU1qWmlORFJpZkdWdUxYVnoiLCJzY2VuYXJpbyI6InNoYXJlTGluayIsImNoYXRUeXBlIjoid2ViIiwicHJvcGVydGllcyI6eyJwcm9tcHRTb3VyY2UiOiJtaWNyb3NvZnQiLCJjbGlja1RpbWVzdGFtcCI6IjIwMjYtMDgtMDhUMjE6MzQ6MTYuODU5WiJ9LCJyZWZlcnJhbCI6eyJjbW1pZCI6ImNtbTEyMjIyMjIyIn0sImNvcnJlbGF0aW9uSWQiOiJjZTc2MmM5Zi04ODM4LTRkMzUtODAxMy0xNDk2OTIzNWEzNGIiLCJ2ZXJzaW9uIjoxLjB9?fromcode=cmm12222222&amp;ct=new&amp;ocid=new&amp;utm_campaign=new&amp;utm_source=new " xr:uid="{4A904F18-ECEF-8E4C-B080-DB124719CDB1}"/>
+    <hyperlink ref="B3" r:id="rId2" display="https://m365.cloud.microsoft/chat/entity1-d870f6cd-4aa5-4d42-9626-ab690c041429/eyJpZCI6IlRXbGpjbTl6YjJaMFZqSjhhSFIwY0hNNkx5OXpkV0p6ZEhKaGRHVXViMlptYVdObExtTnZiWHd5T1dNM04yTmtNeTFsWldJekxUUmhOekV0T1dFelppMDNaRGt6WWpRME9EQXhZako4WlRRMU16RXlaamN0Tm1Fd01DMDBPVFl5TFdGaE0yWXRNekUzWldFMU1qWmlORFJpZkdWdUxYVnoiLCJzY2VuYXJpbyI6InNoYXJlTGluayIsImNoYXRUeXBlIjoid2ViIiwicHJvcGVydGllcyI6eyJwcm9tcHRTb3VyY2UiOiJtaWNyb3NvZnQiLCJjbGlja1RpbWVzdGFtcCI6IjIwMjYtMDgtMDhUMjE6MzQ6MTYuODU5WiJ9LCJyZWZlcnJhbCI6eyJjbW1pZCI6ImNtbTEyMjIyMjIyIn0sImNvcnJlbGF0aW9uSWQiOiJjZTc2MmM5Zi04ODM4LTRkMzUtODAxMy0xNDk2OTIzNWEzNGIiLCJ2ZXJzaW9uIjoxLjB9?fromcode=cmm12222222&amp;ct=new&amp;ocid=new&amp;utm_campaign=new&amp;utm_source=new " xr:uid="{FB00C298-129B-074E-9E51-BE087D0993EF}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Stabilize AppPilot launch flows and logging
</commit_message>
<xml_diff>
--- a/testcases/deeplinks/deeplink_tests.xlsx
+++ b/testcases/deeplinks/deeplink_tests.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10809"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marnisaisanjay/Documents/personalprojects/AppPilot/testcases/deeplinks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95D637E8-0406-0140-8BE7-D18AB3CCDD3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DFD8135-7559-144E-BC9C-86C318ACAE8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{C5943666-9D12-0C47-8784-2B49B0DE6ECC}"/>
   </bookViews>
@@ -539,7 +539,9 @@
   <cols>
     <col min="1" max="1" width="34.6640625" style="1"/>
     <col min="2" max="2" width="138.83203125" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="34.6640625" style="1"/>
+    <col min="3" max="3" width="34.6640625" style="1"/>
+    <col min="4" max="4" width="40.33203125" style="1" customWidth="1"/>
+    <col min="5" max="16384" width="34.6640625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="34" customHeight="1" x14ac:dyDescent="0.2">
@@ -568,7 +570,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:5" s="2" customFormat="1" ht="71" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" s="2" customFormat="1" ht="112" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>11</v>
       </c>
@@ -641,8 +643,8 @@
     <mergeCell ref="A1:E1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B5" r:id="rId1" display="https://m365.cloud.microsoft/chat/entity1-d870f6cd-4aa5-4d42-9626-ab690c041429/eyJpZCI6IlRXbGpjbTl6YjJaMFZqSjhhSFIwY0hNNkx5OXpkV0p6ZEhKaGRHVXViMlptYVdObExtTnZiWHd5T1dNM04yTmtNeTFsWldJekxUUmhOekV0T1dFelppMDNaRGt6WWpRME9EQXhZako4WlRRMU16RXlaamN0Tm1Fd01DMDBPVFl5TFdGaE0yWXRNekUzWldFMU1qWmlORFJpZkdWdUxYVnoiLCJzY2VuYXJpbyI6InNoYXJlTGluayIsImNoYXRUeXBlIjoid2ViIiwicHJvcGVydGllcyI6eyJwcm9tcHRTb3VyY2UiOiJtaWNyb3NvZnQiLCJjbGlja1RpbWVzdGFtcCI6IjIwMjYtMDgtMDhUMjE6MzQ6MTYuODU5WiJ9LCJyZWZlcnJhbCI6eyJjbW1pZCI6ImNtbTEyMjIyMjIyIn0sImNvcnJlbGF0aW9uSWQiOiJjZTc2MmM5Zi04ODM4LTRkMzUtODAxMy0xNDk2OTIzNWEzNGIiLCJ2ZXJzaW9uIjoxLjB9?fromcode=cmm12222222&amp;ct=new&amp;ocid=new&amp;utm_campaign=new&amp;utm_source=new " xr:uid="{4A904F18-ECEF-8E4C-B080-DB124719CDB1}"/>
-    <hyperlink ref="B3" r:id="rId2" display="https://m365.cloud.microsoft/chat/entity1-d870f6cd-4aa5-4d42-9626-ab690c041429/eyJpZCI6IlRXbGpjbTl6YjJaMFZqSjhhSFIwY0hNNkx5OXpkV0p6ZEhKaGRHVXViMlptYVdObExtTnZiWHd5T1dNM04yTmtNeTFsWldJekxUUmhOekV0T1dFelppMDNaRGt6WWpRME9EQXhZako4WlRRMU16RXlaamN0Tm1Fd01DMDBPVFl5TFdGaE0yWXRNekUzWldFMU1qWmlORFJpZkdWdUxYVnoiLCJzY2VuYXJpbyI6InNoYXJlTGluayIsImNoYXRUeXBlIjoid2ViIiwicHJvcGVydGllcyI6eyJwcm9tcHRTb3VyY2UiOiJtaWNyb3NvZnQiLCJjbGlja1RpbWVzdGFtcCI6IjIwMjYtMDgtMDhUMjE6MzQ6MTYuODU5WiJ9LCJyZWZlcnJhbCI6eyJjbW1pZCI6ImNtbTEyMjIyMjIyIn0sImNvcnJlbGF0aW9uSWQiOiJjZTc2MmM5Zi04ODM4LTRkMzUtODAxMy0xNDk2OTIzNWEzNGIiLCJ2ZXJzaW9uIjoxLjB9?fromcode=cmm12222222&amp;ct=new&amp;ocid=new&amp;utm_campaign=new&amp;utm_source=new " xr:uid="{FB00C298-129B-074E-9E51-BE087D0993EF}"/>
+    <hyperlink ref="B3" r:id="rId1" display="https://m365.cloud.microsoft/chat/entity1-d870f6cd-4aa5-4d42-9626-ab690c041429/eyJpZCI6IlRXbGpjbTl6YjJaMFZqSjhhSFIwY0hNNkx5OXpkV0p6ZEhKaGRHVXViMlptYVdObExtTnZiWHd5T1dNM04yTmtNeTFsWldJekxUUmhOekV0T1dFelppMDNaRGt6WWpRME9EQXhZako4WlRRMU16RXlaamN0Tm1Fd01DMDBPVFl5TFdGaE0yWXRNekUzWldFMU1qWmlORFJpZkdWdUxYVnoiLCJzY2VuYXJpbyI6InNoYXJlTGluayIsImNoYXRUeXBlIjoid2ViIiwicHJvcGVydGllcyI6eyJwcm9tcHRTb3VyY2UiOiJtaWNyb3NvZnQiLCJjbGlja1RpbWVzdGFtcCI6IjIwMjYtMDgtMDhUMjE6MzQ6MTYuODU5WiJ9LCJyZWZlcnJhbCI6eyJjbW1pZCI6ImNtbTEyMjIyMjIyIn0sImNvcnJlbGF0aW9uSWQiOiJjZTc2MmM5Zi04ODM4LTRkMzUtODAxMy0xNDk2OTIzNWEzNGIiLCJ2ZXJzaW9uIjoxLjB9?fromcode=cmm12222222&amp;ct=new&amp;ocid=new&amp;utm_campaign=new&amp;utm_source=new " xr:uid="{FB00C298-129B-074E-9E51-BE087D0993EF}"/>
+    <hyperlink ref="B5" r:id="rId2" display="https://m365.cloud.microsoft/chat/entity1-d870f6cd-4aa5-4d42-9626-ab690c041429/eyJpZCI6IlRXbGpjbTl6YjJaMFZqSjhhSFIwY0hNNkx5OXpkV0p6ZEhKaGRHVXViMlptYVdObExtTnZiWHd5T1dNM04yTmtNeTFsWldJekxUUmhOekV0T1dFelppMDNaRGt6WWpRME9EQXhZako4WlRRMU16RXlaamN0Tm1Fd01DMDBPVFl5TFdGaE0yWXRNekUzWldFMU1qWmlORFJpZkdWdUxYVnoiLCJzY2VuYXJpbyI6InNoYXJlTGluayIsImNoYXRUeXBlIjoid2ViIiwicHJvcGVydGllcyI6eyJwcm9tcHRTb3VyY2UiOiJtaWNyb3NvZnQiLCJjbGlja1RpbWVzdGFtcCI6IjIwMjYtMDgtMDhUMjE6MzQ6MTYuODU5WiJ9LCJyZWZlcnJhbCI6eyJjbW1pZCI6ImNtbTEyMjIyMjIyIn0sImNvcnJlbGF0aW9uSWQiOiJjZTc2MmM5Zi04ODM4LTRkMzUtODAxMy0xNDk2OTIzNWEzNGIiLCJ2ZXJzaW9uIjoxLjB9?fromcode=cmm12222222&amp;ct=new&amp;ocid=new&amp;utm_campaign=new&amp;utm_source=new " xr:uid="{4A904F18-ECEF-8E4C-B080-DB124719CDB1}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>